<commit_message>
Correct petrol data source and rounding
</commit_message>
<xml_diff>
--- a/data/petrol_weekly_prices.xlsx
+++ b/data/petrol_weekly_prices.xlsx
@@ -1824,28 +1824,28 @@
         <v>46201</v>
       </c>
       <c r="C44" t="n">
-        <v>160.9</v>
+        <v>155.2</v>
       </c>
       <c r="D44" t="n">
-        <v>170.5</v>
+        <v>167.2</v>
       </c>
       <c r="E44" t="n">
-        <v>163.3</v>
+        <v>157</v>
       </c>
       <c r="F44" t="n">
-        <v>166.1</v>
+        <v>159.2</v>
       </c>
       <c r="G44" t="n">
-        <v>156.9</v>
+        <v>150.7</v>
       </c>
       <c r="H44" t="n">
-        <v>161.7</v>
+        <v>154.8</v>
       </c>
       <c r="I44" t="n">
-        <v>169.3</v>
+        <v>164.7</v>
       </c>
       <c r="J44" t="n">
-        <v>168.7</v>
+        <v>161.8</v>
       </c>
     </row>
     <row r="45">
@@ -1856,28 +1856,28 @@
         <v>46208</v>
       </c>
       <c r="C45" t="n">
-        <v>158.5143</v>
+        <v>158.5</v>
       </c>
       <c r="D45" t="n">
-        <v>169.2429</v>
+        <v>169.2</v>
       </c>
       <c r="E45" t="n">
-        <v>159.9571</v>
+        <v>160</v>
       </c>
       <c r="F45" t="n">
-        <v>160.3571</v>
+        <v>160.4</v>
       </c>
       <c r="G45" t="n">
-        <v>157.4429</v>
+        <v>157.4</v>
       </c>
       <c r="H45" t="n">
         <v>160.9</v>
       </c>
       <c r="I45" t="n">
-        <v>167.6143</v>
+        <v>167.6</v>
       </c>
       <c r="J45" t="n">
-        <v>167.1429</v>
+        <v>167.1</v>
       </c>
     </row>
     <row r="46">
@@ -1888,28 +1888,28 @@
         <v>46215</v>
       </c>
       <c r="C46" t="n">
-        <v>165.5429</v>
+        <v>165.5</v>
       </c>
       <c r="D46" t="n">
-        <v>178.3428</v>
+        <v>178.3</v>
       </c>
       <c r="E46" t="n">
-        <v>166.9429</v>
+        <v>166.9</v>
       </c>
       <c r="F46" t="n">
-        <v>169.8571</v>
+        <v>169.9</v>
       </c>
       <c r="G46" t="n">
-        <v>163.5286</v>
+        <v>163.5</v>
       </c>
       <c r="H46" t="n">
         <v>167.1</v>
       </c>
       <c r="I46" t="n">
-        <v>173.1143</v>
+        <v>173.1</v>
       </c>
       <c r="J46" t="n">
-        <v>173.4286</v>
+        <v>173.4</v>
       </c>
     </row>
     <row r="47">
@@ -1920,28 +1920,28 @@
         <v>46222</v>
       </c>
       <c r="C47" t="n">
-        <v>169.7857</v>
+        <v>169.8</v>
       </c>
       <c r="D47" t="n">
-        <v>178.1286</v>
+        <v>178.1</v>
       </c>
       <c r="E47" t="n">
-        <v>171.5857</v>
+        <v>171.6</v>
       </c>
       <c r="F47" t="n">
-        <v>174.4429</v>
+        <v>174.4</v>
       </c>
       <c r="G47" t="n">
         <v>165.6</v>
       </c>
       <c r="H47" t="n">
-        <v>170.9143</v>
+        <v>170.9</v>
       </c>
       <c r="I47" t="n">
-        <v>175.8143</v>
+        <v>175.8</v>
       </c>
       <c r="J47" t="n">
-        <v>174.1429</v>
+        <v>174.1</v>
       </c>
     </row>
     <row r="48">
@@ -1952,28 +1952,28 @@
         <v>46229</v>
       </c>
       <c r="C48" t="n">
-        <v>178.7286</v>
+        <v>178.7</v>
       </c>
       <c r="D48" t="n">
-        <v>188.2571</v>
+        <v>188.3</v>
       </c>
       <c r="E48" t="n">
-        <v>181.6857</v>
+        <v>181.7</v>
       </c>
       <c r="F48" t="n">
-        <v>183.0286</v>
+        <v>183</v>
       </c>
       <c r="G48" t="n">
-        <v>178.6429</v>
+        <v>178.6</v>
       </c>
       <c r="H48" t="n">
-        <v>180.4857</v>
+        <v>180.5</v>
       </c>
       <c r="I48" t="n">
-        <v>187.0143</v>
+        <v>187</v>
       </c>
       <c r="J48" t="n">
-        <v>184.3428</v>
+        <v>184.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update AIP retail petrol prices
</commit_message>
<xml_diff>
--- a/data/petrol_weekly_prices.xlsx
+++ b/data/petrol_weekly_prices.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1976,6 +1976,38 @@
         <v>184.3</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B49" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C49" t="n">
+        <v>191</v>
+      </c>
+      <c r="D49" t="n">
+        <v>202.1</v>
+      </c>
+      <c r="E49" t="n">
+        <v>193.9</v>
+      </c>
+      <c r="F49" t="n">
+        <v>194.7</v>
+      </c>
+      <c r="G49" t="n">
+        <v>193.1</v>
+      </c>
+      <c r="H49" t="n">
+        <v>191.3</v>
+      </c>
+      <c r="I49" t="n">
+        <v>201.8</v>
+      </c>
+      <c r="J49" t="n">
+        <v>197.1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>